<commit_message>
Separate the live presentation and the rolling program video
- ETLC: "Live Program Presentation" by Dr. Nobes with remarks from the
  MEC E and MCTR clubs, across the stall, schedule, map step, FAQ and
  sticker text.
- Room 3-1: described as a rolling program video (name unchanged, to match
  the printed map); its sticker gets a play button.
- New schedule entry "Rolling program video" (11 AM-2 PM, Room 3-1) under
  Stalls, so the presentation reminder doesn't treat it as a talk.
- The presentation reminder now uses the schedule title, so it follows the
  sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/open-house-content.xlsx
+++ b/content/open-house-content.xlsx
@@ -431,7 +431,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="649">
   <si>
     <t>MEC E Open House website content</t>
   </si>
@@ -610,10 +610,10 @@
     <t>program-presentation</t>
   </si>
   <si>
-    <t>Mechanical Engineering program presentation</t>
-  </si>
-  <si>
-    <t>Learn about the Mechanical Engineering program from the department, with time for questions.</t>
+    <t>Live program presentation</t>
+  </si>
+  <si>
+    <t>Dr. Nobes presents the Mechanical Engineering program, with remarks from the MEC E Club and the Mechatronics (MCTR) Club.</t>
   </si>
   <si>
     <t>10:00</t>
@@ -652,6 +652,21 @@
     <t>2nd and 3rd floors</t>
   </si>
   <si>
+    <t>program-video</t>
+  </si>
+  <si>
+    <t>Rolling program video</t>
+  </si>
+  <si>
+    <t>A short video about the Mechanical Engineering program, playing on a loop. Drop in any time during the building tour.</t>
+  </si>
+  <si>
+    <t>program-room-3-1</t>
+  </si>
+  <si>
+    <t>Room 3-1</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
@@ -733,10 +748,10 @@
     <t>stamp-open-house-booth</t>
   </si>
   <si>
-    <t>MEC E Program Presentation</t>
-  </si>
-  <si>
-    <t>Hear from the department about the Mechanical Engineering program, 10:00 to 11:00 AM in ETLC E1-001.</t>
+    <t>Live Program Presentation</t>
+  </si>
+  <si>
+    <t>A live presentation by Dr. Nobes on the Mechanical Engineering program, with remarks from the MEC E Club and the Mechatronics (MCTR) Club. 10:00 to 11:00 AM in ETLC E1-001.</t>
   </si>
   <si>
     <t>E1-001</t>
@@ -745,7 +760,7 @@
     <t>Program Insider</t>
   </si>
   <si>
-    <t>Collected at the MEC E program presentation.</t>
+    <t>Collected at the live program presentation in ETLC.</t>
   </si>
   <si>
     <t>/assets/stamps/program-presentation.svg</t>
@@ -1320,13 +1335,10 @@
     <t>stamp-mctr-club</t>
   </si>
   <si>
-    <t>program-room-3-1</t>
-  </si>
-  <si>
     <t>Room 3-1: MEC E Program Presentation</t>
   </si>
   <si>
-    <t>Stop by Room 3-1 during the building tour to learn about the Mechanical Engineering program and ask the department your questions.</t>
+    <t>A short video about the Mechanical Engineering program plays on a loop in Room 3-1. Drop in any time during the building tour.</t>
   </si>
   <si>
     <t>3-1</t>
@@ -1335,7 +1347,7 @@
     <t>Program Preview</t>
   </si>
   <si>
-    <t>Collected in Room 3-1 on the building tour.</t>
+    <t>Collected at the program video in Room 3-1.</t>
   </si>
   <si>
     <t>/assets/stamps/program-room-3-1.svg</t>
@@ -1425,7 +1437,7 @@
     <t>When and where is the Open House?</t>
   </si>
   <si>
-    <t>Saturday, October 17, 2026, from 9:00 AM to 3:00 PM. Start at the Mechanical Engineering stall in the VVC gym, catch the program presentation at 10:00 AM in ETLC E1-001, then tour the Mechanical Engineering Building from 11:00 AM to 2:00 PM. The Map page shows the way.</t>
+    <t>Saturday, October 17, 2026, from 9:00 AM to 3:00 PM. Start at the Mechanical Engineering stall in the VVC gym, catch the live program presentation with Dr. Nobes at 10:00 AM in ETLC E1-001, then tour the Mechanical Engineering Building from 11:00 AM to 2:00 PM. The Map page shows the way.</t>
   </si>
   <si>
     <t>register</t>
@@ -3035,7 +3047,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K203"/>
+  <dimension ref="A1:K204"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" style="7" customWidth="1"/>
@@ -3185,9 +3197,40 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="6:11" x14ac:dyDescent="0.25">
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+    <row r="5" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="6" spans="6:11" x14ac:dyDescent="0.25">
       <c r="F6" s="7"/>
@@ -3981,24 +4024,28 @@
       <c r="F203" s="7"/>
       <c r="G203" s="7"/>
     </row>
+    <row r="204" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F204" s="7"/>
+      <c r="G204" s="7"/>
+    </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" sqref="F10:F203">
+    <dataValidation type="list" allowBlank="1" sqref="F10:F204">
       <formula1>"presentation,tour,booth-fair,food,general"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F203">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F204">
       <formula1>"presentation,tour,booth-fair,food,general"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G10:G203">
+    <dataValidation type="list" allowBlank="1" sqref="G10:G204">
       <formula1>"mece,university"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G203">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G204">
       <formula1>"mece,university"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K10:K203">
+    <dataValidation type="list" allowBlank="1" sqref="K10:K204">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K2:K203">
+    <dataValidation type="list" allowBlank="1" sqref="K2:K204">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4036,61 +4083,61 @@
         <v>39</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>46</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="T1" s="11" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4098,16 +4145,16 @@
         <v>55</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F2" s="9"/>
       <c r="G2" s="5"/>
@@ -4123,28 +4170,28 @@
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="M2" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="R2" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="T2" s="12" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4152,16 +4199,16 @@
         <v>58</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>63</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="5"/>
@@ -4172,33 +4219,33 @@
         <v>1</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="P3" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="R3" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4206,16 +4253,16 @@
         <v>71</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="5"/>
@@ -4226,7 +4273,7 @@
         <v>2</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="K4" s="9">
         <v>0.236</v>
@@ -4235,45 +4282,45 @@
         <v>0.349</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="P4" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="R4" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="5"/>
@@ -4284,7 +4331,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K5" s="9">
         <v>0.372</v>
@@ -4293,51 +4340,51 @@
         <v>0.498</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="P5" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="R5" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>34</v>
@@ -4346,7 +4393,7 @@
         <v>3</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="K6" s="9">
         <v>0.805</v>
@@ -4355,49 +4402,49 @@
         <v>0.66</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="P6" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R6" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="T6" s="12" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>34</v>
@@ -4406,7 +4453,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="K7" s="9">
         <v>0.684</v>
@@ -4415,51 +4462,51 @@
         <v>0.763</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="P7" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="R7" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="T7" s="12" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>34</v>
@@ -4468,7 +4515,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K8" s="9">
         <v>0.275</v>
@@ -4477,45 +4524,45 @@
         <v>0.598</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="P8" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="R8" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S8" s="12" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="T8" s="12" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="5"/>
@@ -4526,7 +4573,7 @@
         <v>3</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K9" s="9">
         <v>0.714</v>
@@ -4535,45 +4582,45 @@
         <v>0.491</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="P9" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R9" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="T9" s="12" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="5"/>
@@ -4584,7 +4631,7 @@
         <v>3</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="K10" s="9">
         <v>0.513</v>
@@ -4593,49 +4640,49 @@
         <v>0.67</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="P10" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="R10" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S10" s="12" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="T10" s="12" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -4644,7 +4691,7 @@
         <v>3</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K11" s="9">
         <v>0.29</v>
@@ -4653,49 +4700,49 @@
         <v>0.566</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="P11" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="R11" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S11" s="12" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="T11" s="12" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>34</v>
@@ -4704,7 +4751,7 @@
         <v>3</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K12" s="9">
         <v>0.159</v>
@@ -4713,51 +4760,51 @@
         <v>0.649</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="P12" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="R12" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="T12" s="12" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>34</v>
@@ -4766,7 +4813,7 @@
         <v>3</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K13" s="9">
         <v>0.161</v>
@@ -4775,49 +4822,49 @@
         <v>0.651</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="R13" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S13" s="12" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="T13" s="12" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>34</v>
@@ -4826,7 +4873,7 @@
         <v>3</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K14" s="9">
         <v>0.245</v>
@@ -4835,45 +4882,45 @@
         <v>0.571</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="P14" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="R14" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S14" s="12" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="T14" s="12" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="15" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="5"/>
@@ -4884,7 +4931,7 @@
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="K15" s="9">
         <v>0.153</v>
@@ -4893,49 +4940,49 @@
         <v>0.164</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="P15" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="R15" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S15" s="12" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="T15" s="12" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="5" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>34</v>
@@ -4944,7 +4991,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="K16" s="9">
         <v>0.685</v>
@@ -4953,49 +5000,49 @@
         <v>0.758</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="P16" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="R16" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S16" s="12" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="T16" s="12" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="5" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>34</v>
@@ -5004,7 +5051,7 @@
         <v>3</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="K17" s="9">
         <v>0.285</v>
@@ -5013,49 +5060,49 @@
         <v>0.571</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="R17" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="T17" s="12" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>34</v>
@@ -5064,7 +5111,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="K18" s="9">
         <v>0.66</v>
@@ -5073,49 +5120,49 @@
         <v>0.603</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="P18" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="R18" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S18" s="12" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="T18" s="12" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>34</v>
@@ -5124,7 +5171,7 @@
         <v>3</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="K19" s="9">
         <v>0.233</v>
@@ -5133,45 +5180,45 @@
         <v>0.343</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="P19" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="R19" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S19" s="12" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="T19" s="12" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="20" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>295</v>
+        <v>76</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>63</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="5"/>
@@ -5182,7 +5229,7 @@
         <v>3</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="K20" s="9">
         <v>0.271</v>
@@ -5191,28 +5238,28 @@
         <v>0.817</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="R20" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21" spans="3:18" x14ac:dyDescent="0.25">
@@ -5853,7 +5900,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -5861,111 +5908,111 @@
         <v>71</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>295</v>
+        <v>76</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -5996,39 +6043,39 @@
         <v>44</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -6042,16 +6089,16 @@
     </row>
     <row r="3" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
@@ -6065,16 +6112,16 @@
     </row>
     <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
@@ -6088,16 +6135,16 @@
     </row>
     <row r="5" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
@@ -6111,23 +6158,23 @@
     </row>
     <row r="6" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="5" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>30</v>
@@ -6138,20 +6185,20 @@
     </row>
     <row r="7" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="9" t="s">
@@ -6163,16 +6210,16 @@
     </row>
     <row r="8" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
@@ -6186,16 +6233,16 @@
     </row>
     <row r="9" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
@@ -6209,16 +6256,16 @@
     </row>
     <row r="10" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
@@ -6232,16 +6279,16 @@
     </row>
     <row r="11" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
@@ -6255,23 +6302,23 @@
     </row>
     <row r="12" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>30</v>
@@ -6282,16 +6329,16 @@
     </row>
     <row r="13" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
@@ -6305,16 +6352,16 @@
     </row>
     <row r="14" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
@@ -6328,16 +6375,16 @@
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
@@ -6351,16 +6398,16 @@
     </row>
     <row r="16" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
@@ -6374,16 +6421,16 @@
     </row>
     <row r="17" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
@@ -6397,23 +6444,23 @@
     </row>
     <row r="18" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>30</v>
@@ -6657,46 +6704,46 @@
         <v>44</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G2" s="9">
         <v>53.523554</v>
@@ -6711,20 +6758,20 @@
     </row>
     <row r="3" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G3" s="9">
         <v>53.521287</v>
@@ -6739,20 +6786,20 @@
     </row>
     <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>403</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>399</v>
       </c>
       <c r="G4" s="9">
         <v>53.528897</v>
@@ -6767,20 +6814,20 @@
     </row>
     <row r="5" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G5" s="9">
         <v>53.526203</v>
@@ -6795,20 +6842,20 @@
     </row>
     <row r="6" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G6" s="9">
         <v>53.52527</v>
@@ -6823,20 +6870,20 @@
     </row>
     <row r="7" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G7" s="9">
         <v>53.525312</v>
@@ -6851,20 +6898,20 @@
     </row>
     <row r="8" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="G8" s="9">
         <v>53.528827</v>
@@ -6879,20 +6926,20 @@
     </row>
     <row r="9" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="G9" s="9">
         <v>53.525374</v>
@@ -6907,20 +6954,20 @@
     </row>
     <row r="10" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="G10" s="9">
         <v>53.52575</v>
@@ -6935,20 +6982,20 @@
     </row>
     <row r="11" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="G11" s="9">
         <v>53.526227</v>
@@ -6963,20 +7010,20 @@
     </row>
     <row r="12" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="G12" s="9">
         <v>53.521933</v>
@@ -6991,20 +7038,20 @@
     </row>
     <row r="13" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="G13" s="9">
         <v>53.526054</v>
@@ -7019,20 +7066,20 @@
     </row>
     <row r="14" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G14" s="9">
         <v>53.527982</v>
@@ -7047,20 +7094,20 @@
     </row>
     <row r="15" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G15" s="9">
         <v>53.526848</v>
@@ -7075,20 +7122,20 @@
     </row>
     <row r="16" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G16" s="9">
         <v>53.518596</v>
@@ -7103,20 +7150,20 @@
     </row>
     <row r="17" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="G17" s="9">
         <v>53.525281</v>
@@ -7131,20 +7178,20 @@
     </row>
     <row r="18" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="G18" s="9">
         <v>53.526405</v>
@@ -7159,20 +7206,20 @@
     </row>
     <row r="19" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G19" s="9">
         <v>53.526452</v>
@@ -7189,20 +7236,20 @@
     </row>
     <row r="20" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G20" s="9">
         <v>53.520234</v>
@@ -7219,20 +7266,20 @@
     </row>
     <row r="21" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G21" s="9">
         <v>53.526721</v>
@@ -7249,20 +7296,20 @@
     </row>
     <row r="22" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G22" s="9">
         <v>53.522632</v>
@@ -7279,20 +7326,20 @@
     </row>
     <row r="23" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G23" s="9">
         <v>53.520485</v>
@@ -7309,20 +7356,20 @@
     </row>
     <row r="24" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G24" s="9">
         <v>53.526051</v>
@@ -7339,20 +7386,20 @@
     </row>
     <row r="25" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G25" s="9">
         <v>53.526912</v>
@@ -7369,20 +7416,20 @@
     </row>
     <row r="26" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G26" s="9">
         <v>53.519489</v>
@@ -7399,20 +7446,20 @@
     </row>
     <row r="27" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="G27" s="9">
         <v>53.526097</v>
@@ -7429,20 +7476,20 @@
     </row>
     <row r="28" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G28" s="9">
         <v>53.522735</v>
@@ -7459,20 +7506,20 @@
     </row>
     <row r="29" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G29" s="9">
         <v>53.523398</v>
@@ -7489,20 +7536,20 @@
     </row>
     <row r="30" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G30" s="9">
         <v>53.526831</v>
@@ -7519,20 +7566,20 @@
     </row>
     <row r="31" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G31" s="9">
         <v>53.522498</v>
@@ -7549,20 +7596,20 @@
     </row>
     <row r="32" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G32" s="9">
         <v>53.521206</v>
@@ -7579,20 +7626,20 @@
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G33" s="9">
         <v>53.526778</v>
@@ -7609,20 +7656,20 @@
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G34" s="9">
         <v>53.521769</v>
@@ -7639,20 +7686,20 @@
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G35" s="9">
         <v>53.527243</v>
@@ -7669,20 +7716,20 @@
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G36" s="9">
         <v>53.526834</v>
@@ -7699,20 +7746,20 @@
     </row>
     <row r="37" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G37" s="9">
         <v>53.521291</v>
@@ -7729,20 +7776,20 @@
     </row>
     <row r="38" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G38" s="9">
         <v>53.526281</v>
@@ -7759,20 +7806,20 @@
     </row>
     <row r="39" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G39" s="9">
         <v>53.527298</v>
@@ -7789,20 +7836,20 @@
     </row>
     <row r="40" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G40" s="9">
         <v>53.526922</v>
@@ -7819,20 +7866,20 @@
     </row>
     <row r="41" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="G41" s="9">
         <v>53.525208</v>
@@ -7849,20 +7896,20 @@
     </row>
     <row r="42" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G42" s="9">
         <v>53.527654</v>
@@ -7879,20 +7926,20 @@
     </row>
     <row r="43" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G43" s="9">
         <v>53.529014</v>
@@ -7909,20 +7956,20 @@
     </row>
     <row r="44" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G44" s="9">
         <v>53.521611</v>
@@ -7939,20 +7986,20 @@
     </row>
     <row r="45" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="G45" s="9">
         <v>53.521595</v>
@@ -7969,20 +8016,20 @@
     </row>
     <row r="46" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G46" s="9">
         <v>53.520763</v>
@@ -7999,20 +8046,20 @@
     </row>
     <row r="47" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G47" s="9">
         <v>53.526621</v>
@@ -8029,20 +8076,20 @@
     </row>
     <row r="48" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G48" s="9">
         <v>53.521375</v>
@@ -8059,20 +8106,20 @@
     </row>
     <row r="49" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G49" s="9">
         <v>53.525055</v>
@@ -8089,20 +8136,20 @@
     </row>
     <row r="50" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="G50" s="9">
         <v>53.522628</v>
@@ -8119,20 +8166,20 @@
     </row>
     <row r="51" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G51" s="9">
         <v>53.52057</v>
@@ -8149,20 +8196,20 @@
     </row>
     <row r="52" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G52" s="9">
         <v>53.527441</v>
@@ -8179,20 +8226,20 @@
     </row>
     <row r="53" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G53" s="9">
         <v>53.521685</v>
@@ -8209,20 +8256,20 @@
     </row>
     <row r="54" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G54" s="9">
         <v>53.52063</v>
@@ -8239,20 +8286,20 @@
     </row>
     <row r="55" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="G55" s="9">
         <v>53.52495</v>
@@ -8267,20 +8314,20 @@
     </row>
     <row r="56" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B56" s="5" t="s">
         <v>523</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>519</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="G56" s="9">
         <v>53.52455</v>
@@ -8295,20 +8342,20 @@
     </row>
     <row r="57" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="G57" s="9">
         <v>53.51885</v>
@@ -8323,20 +8370,20 @@
     </row>
     <row r="58" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="G58" s="9">
         <v>53.52735</v>
@@ -8351,20 +8398,20 @@
     </row>
     <row r="59" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="G59" s="9">
         <v>53.520064</v>
@@ -8379,20 +8426,20 @@
     </row>
     <row r="60" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C60" s="5"/>
       <c r="D60" s="5" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="G60" s="9">
         <v>53.52485</v>
@@ -8407,22 +8454,22 @@
     </row>
     <row r="61" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="G61" s="9">
         <v>53.524907</v>
@@ -8439,22 +8486,22 @@
     </row>
     <row r="62" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C62" s="5" t="s">
         <v>547</v>
       </c>
-      <c r="B62" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>543</v>
-      </c>
       <c r="D62" s="5" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="G62" s="9">
         <v>53.524349</v>
@@ -8471,22 +8518,22 @@
     </row>
     <row r="63" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="G63" s="9">
         <v>53.522853</v>
@@ -8503,22 +8550,22 @@
     </row>
     <row r="64" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="G64" s="9">
         <v>53.522936</v>
@@ -8535,22 +8582,22 @@
     </row>
     <row r="65" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="G65" s="9">
         <v>53.522841</v>
@@ -8567,22 +8614,22 @@
     </row>
     <row r="66" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="G66" s="9">
         <v>53.527555</v>
@@ -8599,22 +8646,22 @@
     </row>
     <row r="67" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="G67" s="9">
         <v>53.526058</v>
@@ -8631,22 +8678,22 @@
     </row>
     <row r="68" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="G68" s="9">
         <v>53.520408</v>
@@ -8663,22 +8710,22 @@
     </row>
     <row r="69" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="G69" s="9">
         <v>53.521436</v>
@@ -8695,22 +8742,22 @@
     </row>
     <row r="70" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="G70" s="9">
         <v>53.520333</v>
@@ -8727,22 +8774,22 @@
     </row>
     <row r="71" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="G71" s="9">
         <v>53.522316</v>
@@ -8759,22 +8806,22 @@
     </row>
     <row r="72" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="G72" s="9">
         <v>53.522998</v>
@@ -8791,22 +8838,22 @@
     </row>
     <row r="73" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="G73" s="9">
         <v>53.519823</v>
@@ -8823,22 +8870,22 @@
     </row>
     <row r="74" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="G74" s="9">
         <v>53.518952</v>
@@ -8855,22 +8902,22 @@
     </row>
     <row r="75" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="G75" s="9">
         <v>53.521462</v>
@@ -8887,22 +8934,22 @@
     </row>
     <row r="76" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="G76" s="9">
         <v>53.522356</v>
@@ -8919,22 +8966,22 @@
     </row>
     <row r="77" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="G77" s="9">
         <v>53.523026</v>
@@ -8951,22 +8998,22 @@
     </row>
     <row r="78" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="G78" s="9">
         <v>53.524645</v>
@@ -8983,22 +9030,22 @@
     </row>
     <row r="79" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="G79" s="9">
         <v>53.522775</v>
@@ -9015,22 +9062,22 @@
     </row>
     <row r="80" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="G80" s="9">
         <v>53.523038</v>
@@ -9047,22 +9094,22 @@
     </row>
     <row r="81" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="G81" s="9">
         <v>53.519278</v>
@@ -9079,22 +9126,22 @@
     </row>
     <row r="82" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="G82" s="9">
         <v>53.52115</v>
@@ -9111,22 +9158,22 @@
     </row>
     <row r="83" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="G83" s="9">
         <v>53.522884</v>
@@ -9143,22 +9190,22 @@
     </row>
     <row r="84" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="G84" s="9">
         <v>53.520281</v>
@@ -9175,22 +9222,22 @@
     </row>
     <row r="85" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="G85" s="9">
         <v>53.522781</v>
@@ -9207,22 +9254,22 @@
     </row>
     <row r="86" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="G86" s="9">
         <v>53.52484</v>
@@ -9239,22 +9286,22 @@
     </row>
     <row r="87" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="G87" s="9">
         <v>53.524712</v>
@@ -9271,22 +9318,22 @@
     </row>
     <row r="88" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="G88" s="9">
         <v>53.524751</v>

</xml_diff>

<commit_message>
Password-protect the QR codes page
/qr-codes asks for a password before showing any code. Only a salted
SHA-256 fingerprint is stored (event.json -> qrPagePasswordHash), never the
password. Change it on the content sheet's Event tab ("QR codes page
password"; blank keeps the current one) or with
`npm run qr:password -- "new password"`. The unlock lasts for the browser
tab and a new password locks it again.

This is a light lock: the stall codes themselves are still in the site's
files until codes are checked by a server.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/open-house-content.xlsx
+++ b/content/open-house-content.xlsx
@@ -431,7 +431,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="647">
   <si>
     <t>MEC E Open House website content</t>
   </si>
@@ -530,6 +530,12 @@
   </si>
   <si>
     <t>Optional. Adds a 'MEC E programs calendar' card</t>
+  </si>
+  <si>
+    <t>QR codes page password</t>
+  </si>
+  <si>
+    <t>Type a new password to change it (8+ characters). Leave blank to keep the current one. Only a fingerprint is stored on the website</t>
   </si>
   <si>
     <t>Tour building ID</t>
@@ -2895,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2993,32 +2999,41 @@
       <c r="A9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="5"/>
+      <c r="C9" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="5">
-        <v>1</v>
-      </c>
       <c r="C10" s="6" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="5" t="s">
         <v>38</v>
       </c>
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
       <c r="C11" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3047,48 +3062,48 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>24</v>
@@ -3097,92 +3112,92 @@
         <v>27</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="6:11" x14ac:dyDescent="0.25">
@@ -4033,200 +4048,200 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="T1" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F2" s="9"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" s="9">
         <v>1</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="M2" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="R2" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="T2" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I3" s="9">
         <v>1</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="P3" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" s="9">
         <v>2</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K4" s="9">
         <v>0.236</v>
@@ -4235,56 +4250,56 @@
         <v>0.349</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P4" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I5" s="9">
         <v>2</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K5" s="9">
         <v>0.372</v>
@@ -4293,60 +4308,60 @@
         <v>0.498</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P5" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="R5" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I6" s="9">
         <v>3</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K6" s="9">
         <v>0.805</v>
@@ -4355,58 +4370,58 @@
         <v>0.66</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P6" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="T6" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I7" s="9">
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K7" s="9">
         <v>0.684</v>
@@ -4415,60 +4430,60 @@
         <v>0.763</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="R7" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="T7" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I8" s="9">
         <v>2</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K8" s="9">
         <v>0.275</v>
@@ -4477,56 +4492,56 @@
         <v>0.598</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="P8" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="R8" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S8" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T8" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I9" s="9">
         <v>3</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="K9" s="9">
         <v>0.714</v>
@@ -4535,56 +4550,56 @@
         <v>0.491</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="P9" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="R9" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="T9" s="12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I10" s="9">
         <v>3</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="K10" s="9">
         <v>0.513</v>
@@ -4593,58 +4608,58 @@
         <v>0.67</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="P10" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S10" s="12" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="T10" s="12" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I11" s="9">
         <v>3</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K11" s="9">
         <v>0.29</v>
@@ -4653,58 +4668,58 @@
         <v>0.566</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="R11" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S11" s="12" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="T11" s="12" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I12" s="9">
         <v>3</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K12" s="9">
         <v>0.159</v>
@@ -4713,60 +4728,60 @@
         <v>0.649</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="P12" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="R12" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="T12" s="12" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I13" s="9">
         <v>3</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K13" s="9">
         <v>0.161</v>
@@ -4775,58 +4790,58 @@
         <v>0.651</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="R13" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S13" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="T13" s="12" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I14" s="9">
         <v>3</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K14" s="9">
         <v>0.245</v>
@@ -4835,56 +4850,56 @@
         <v>0.571</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="P14" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="R14" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S14" s="12" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="T14" s="12" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I15" s="9">
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="K15" s="9">
         <v>0.153</v>
@@ -4893,58 +4908,58 @@
         <v>0.164</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="P15" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="R15" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S15" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="T15" s="12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I16" s="9">
         <v>2</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K16" s="9">
         <v>0.685</v>
@@ -4953,58 +4968,58 @@
         <v>0.758</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="P16" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="R16" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S16" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="T16" s="12" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I17" s="9">
         <v>3</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K17" s="9">
         <v>0.285</v>
@@ -5013,58 +5028,58 @@
         <v>0.571</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="T17" s="12" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I18" s="9">
         <v>2</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K18" s="9">
         <v>0.66</v>
@@ -5073,58 +5088,58 @@
         <v>0.603</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="P18" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="R18" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S18" s="12" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="T18" s="12" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I19" s="9">
         <v>3</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="K19" s="9">
         <v>0.233</v>
@@ -5133,56 +5148,56 @@
         <v>0.343</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="R19" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S19" s="12" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="T19" s="12" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I20" s="9">
         <v>3</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K20" s="9">
         <v>0.271</v>
@@ -5191,28 +5206,28 @@
         <v>0.817</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="R20" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="21" spans="3:18" x14ac:dyDescent="0.25">
@@ -5850,122 +5865,122 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -5990,45 +6005,45 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -6042,16 +6057,16 @@
     </row>
     <row r="3" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
@@ -6065,16 +6080,16 @@
     </row>
     <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
@@ -6088,16 +6103,16 @@
     </row>
     <row r="5" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
@@ -6111,23 +6126,23 @@
     </row>
     <row r="6" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="5" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>30</v>
@@ -6138,20 +6153,20 @@
     </row>
     <row r="7" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="9" t="s">
@@ -6163,16 +6178,16 @@
     </row>
     <row r="8" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
@@ -6186,16 +6201,16 @@
     </row>
     <row r="9" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
@@ -6209,16 +6224,16 @@
     </row>
     <row r="10" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
@@ -6227,21 +6242,21 @@
         <v>30</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
@@ -6255,23 +6270,23 @@
     </row>
     <row r="12" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>30</v>
@@ -6282,16 +6297,16 @@
     </row>
     <row r="13" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
@@ -6305,16 +6320,16 @@
     </row>
     <row r="14" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
@@ -6328,16 +6343,16 @@
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
@@ -6346,21 +6361,21 @@
         <v>30</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
@@ -6374,16 +6389,16 @@
     </row>
     <row r="17" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
@@ -6397,23 +6412,23 @@
     </row>
     <row r="18" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>30</v>
@@ -6651,52 +6666,52 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G2" s="9">
         <v>53.523554</v>
@@ -6711,20 +6726,20 @@
     </row>
     <row r="3" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>401</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>399</v>
       </c>
       <c r="G3" s="9">
         <v>53.521287</v>
@@ -6739,20 +6754,20 @@
     </row>
     <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G4" s="9">
         <v>53.528897</v>
@@ -6767,20 +6782,20 @@
     </row>
     <row r="5" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G5" s="9">
         <v>53.526203</v>
@@ -6795,20 +6810,20 @@
     </row>
     <row r="6" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G6" s="9">
         <v>53.52527</v>
@@ -6823,20 +6838,20 @@
     </row>
     <row r="7" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G7" s="9">
         <v>53.525312</v>
@@ -6851,20 +6866,20 @@
     </row>
     <row r="8" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G8" s="9">
         <v>53.528827</v>
@@ -6879,20 +6894,20 @@
     </row>
     <row r="9" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="G9" s="9">
         <v>53.525374</v>
@@ -6901,26 +6916,26 @@
         <v>-113.524077</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J9" s="9"/>
     </row>
     <row r="10" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="G10" s="9">
         <v>53.52575</v>
@@ -6929,26 +6944,26 @@
         <v>-113.52365</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J10" s="9"/>
     </row>
     <row r="11" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G11" s="9">
         <v>53.526227</v>
@@ -6957,26 +6972,26 @@
         <v>-113.520488</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J11" s="9"/>
     </row>
     <row r="12" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="G12" s="9">
         <v>53.521933</v>
@@ -6985,26 +7000,26 @@
         <v>-113.530584</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J12" s="9"/>
     </row>
     <row r="13" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>427</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>425</v>
       </c>
       <c r="G13" s="9">
         <v>53.526054</v>
@@ -7013,26 +7028,26 @@
         <v>-113.516925</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J13" s="9"/>
     </row>
     <row r="14" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G14" s="9">
         <v>53.527982</v>
@@ -7041,26 +7056,26 @@
         <v>-113.526094</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J14" s="9"/>
     </row>
     <row r="15" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>434</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>432</v>
       </c>
       <c r="G15" s="9">
         <v>53.526848</v>
@@ -7069,26 +7084,26 @@
         <v>-113.524059</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J15" s="9"/>
     </row>
     <row r="16" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G16" s="9">
         <v>53.518596</v>
@@ -7097,26 +7112,26 @@
         <v>-113.520352</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G17" s="9">
         <v>53.525281</v>
@@ -7125,26 +7140,26 @@
         <v>-113.527125</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J17" s="9"/>
     </row>
     <row r="18" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="G18" s="9">
         <v>53.526405</v>
@@ -7153,26 +7168,26 @@
         <v>-113.524923</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J18" s="9"/>
     </row>
     <row r="19" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G19" s="9">
         <v>53.526452</v>
@@ -7189,20 +7204,20 @@
     </row>
     <row r="20" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>449</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>449</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>447</v>
       </c>
       <c r="G20" s="9">
         <v>53.520234</v>
@@ -7219,20 +7234,20 @@
     </row>
     <row r="21" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G21" s="9">
         <v>53.526721</v>
@@ -7249,20 +7264,20 @@
     </row>
     <row r="22" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G22" s="9">
         <v>53.522632</v>
@@ -7279,20 +7294,20 @@
     </row>
     <row r="23" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G23" s="9">
         <v>53.520485</v>
@@ -7309,20 +7324,20 @@
     </row>
     <row r="24" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G24" s="9">
         <v>53.526051</v>
@@ -7339,20 +7354,20 @@
     </row>
     <row r="25" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G25" s="9">
         <v>53.526912</v>
@@ -7369,20 +7384,20 @@
     </row>
     <row r="26" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G26" s="9">
         <v>53.519489</v>
@@ -7399,20 +7414,20 @@
     </row>
     <row r="27" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G27" s="9">
         <v>53.526097</v>
@@ -7429,20 +7444,20 @@
     </row>
     <row r="28" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G28" s="9">
         <v>53.522735</v>
@@ -7459,20 +7474,20 @@
     </row>
     <row r="29" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G29" s="9">
         <v>53.523398</v>
@@ -7489,20 +7504,20 @@
     </row>
     <row r="30" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G30" s="9">
         <v>53.526831</v>
@@ -7519,20 +7534,20 @@
     </row>
     <row r="31" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G31" s="9">
         <v>53.522498</v>
@@ -7549,20 +7564,20 @@
     </row>
     <row r="32" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G32" s="9">
         <v>53.521206</v>
@@ -7579,20 +7594,20 @@
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G33" s="9">
         <v>53.526778</v>
@@ -7609,20 +7624,20 @@
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G34" s="9">
         <v>53.521769</v>
@@ -7639,20 +7654,20 @@
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G35" s="9">
         <v>53.527243</v>
@@ -7669,20 +7684,20 @@
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G36" s="9">
         <v>53.526834</v>
@@ -7699,20 +7714,20 @@
     </row>
     <row r="37" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G37" s="9">
         <v>53.521291</v>
@@ -7729,20 +7744,20 @@
     </row>
     <row r="38" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G38" s="9">
         <v>53.526281</v>
@@ -7759,20 +7774,20 @@
     </row>
     <row r="39" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G39" s="9">
         <v>53.527298</v>
@@ -7789,20 +7804,20 @@
     </row>
     <row r="40" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G40" s="9">
         <v>53.526922</v>
@@ -7819,20 +7834,20 @@
     </row>
     <row r="41" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G41" s="9">
         <v>53.525208</v>
@@ -7849,20 +7864,20 @@
     </row>
     <row r="42" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G42" s="9">
         <v>53.527654</v>
@@ -7879,20 +7894,20 @@
     </row>
     <row r="43" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G43" s="9">
         <v>53.529014</v>
@@ -7909,20 +7924,20 @@
     </row>
     <row r="44" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G44" s="9">
         <v>53.521611</v>
@@ -7939,20 +7954,20 @@
     </row>
     <row r="45" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G45" s="9">
         <v>53.521595</v>
@@ -7969,20 +7984,20 @@
     </row>
     <row r="46" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G46" s="9">
         <v>53.520763</v>
@@ -7999,20 +8014,20 @@
     </row>
     <row r="47" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G47" s="9">
         <v>53.526621</v>
@@ -8029,20 +8044,20 @@
     </row>
     <row r="48" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G48" s="9">
         <v>53.521375</v>
@@ -8059,20 +8074,20 @@
     </row>
     <row r="49" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G49" s="9">
         <v>53.525055</v>
@@ -8089,20 +8104,20 @@
     </row>
     <row r="50" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G50" s="9">
         <v>53.522628</v>
@@ -8119,20 +8134,20 @@
     </row>
     <row r="51" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G51" s="9">
         <v>53.52057</v>
@@ -8149,20 +8164,20 @@
     </row>
     <row r="52" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G52" s="9">
         <v>53.527441</v>
@@ -8179,20 +8194,20 @@
     </row>
     <row r="53" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G53" s="9">
         <v>53.521685</v>
@@ -8209,20 +8224,20 @@
     </row>
     <row r="54" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G54" s="9">
         <v>53.52063</v>
@@ -8239,20 +8254,20 @@
     </row>
     <row r="55" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="G55" s="9">
         <v>53.52495</v>
@@ -8267,20 +8282,20 @@
     </row>
     <row r="56" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G56" s="9">
         <v>53.52455</v>
@@ -8295,20 +8310,20 @@
     </row>
     <row r="57" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="G57" s="9">
         <v>53.51885</v>
@@ -8323,20 +8338,20 @@
     </row>
     <row r="58" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="G58" s="9">
         <v>53.52735</v>
@@ -8351,20 +8366,20 @@
     </row>
     <row r="59" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="G59" s="9">
         <v>53.520064</v>
@@ -8379,20 +8394,20 @@
     </row>
     <row r="60" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C60" s="5"/>
       <c r="D60" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="F60" s="5" t="s">
         <v>540</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>541</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>538</v>
       </c>
       <c r="G60" s="9">
         <v>53.52485</v>
@@ -8407,22 +8422,22 @@
     </row>
     <row r="61" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="G61" s="9">
         <v>53.524907</v>
@@ -8439,22 +8454,22 @@
     </row>
     <row r="62" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="G62" s="9">
         <v>53.524349</v>
@@ -8471,22 +8486,22 @@
     </row>
     <row r="63" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G63" s="9">
         <v>53.522853</v>
@@ -8503,22 +8518,22 @@
     </row>
     <row r="64" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="G64" s="9">
         <v>53.522936</v>
@@ -8535,22 +8550,22 @@
     </row>
     <row r="65" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="G65" s="9">
         <v>53.522841</v>
@@ -8567,22 +8582,22 @@
     </row>
     <row r="66" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="G66" s="9">
         <v>53.527555</v>
@@ -8599,22 +8614,22 @@
     </row>
     <row r="67" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="G67" s="9">
         <v>53.526058</v>
@@ -8631,22 +8646,22 @@
     </row>
     <row r="68" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="G68" s="9">
         <v>53.520408</v>
@@ -8663,22 +8678,22 @@
     </row>
     <row r="69" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="G69" s="9">
         <v>53.521436</v>
@@ -8695,22 +8710,22 @@
     </row>
     <row r="70" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="G70" s="9">
         <v>53.520333</v>
@@ -8727,22 +8742,22 @@
     </row>
     <row r="71" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="G71" s="9">
         <v>53.522316</v>
@@ -8759,22 +8774,22 @@
     </row>
     <row r="72" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
+        <v>589</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="E72" s="5" t="s">
         <v>587</v>
       </c>
-      <c r="B72" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>584</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>585</v>
-      </c>
       <c r="F72" s="5" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="G72" s="9">
         <v>53.522998</v>
@@ -8791,22 +8806,22 @@
     </row>
     <row r="73" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="G73" s="9">
         <v>53.519823</v>
@@ -8823,22 +8838,22 @@
     </row>
     <row r="74" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>593</v>
       </c>
-      <c r="B74" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>590</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>591</v>
-      </c>
       <c r="F74" s="5" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="G74" s="9">
         <v>53.518952</v>
@@ -8855,22 +8870,22 @@
     </row>
     <row r="75" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="G75" s="9">
         <v>53.521462</v>
@@ -8887,22 +8902,22 @@
     </row>
     <row r="76" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="G76" s="9">
         <v>53.522356</v>
@@ -8919,22 +8934,22 @@
     </row>
     <row r="77" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
+        <v>605</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>603</v>
       </c>
-      <c r="B77" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C77" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>600</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>601</v>
-      </c>
       <c r="F77" s="5" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="G77" s="9">
         <v>53.523026</v>
@@ -8951,22 +8966,22 @@
     </row>
     <row r="78" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="G78" s="9">
         <v>53.524645</v>
@@ -8983,22 +8998,22 @@
     </row>
     <row r="79" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G79" s="9">
         <v>53.522775</v>
@@ -9015,22 +9030,22 @@
     </row>
     <row r="80" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="E80" s="5" t="s">
         <v>613</v>
       </c>
-      <c r="B80" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C80" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>610</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>611</v>
-      </c>
       <c r="F80" s="5" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="G80" s="9">
         <v>53.523038</v>
@@ -9047,22 +9062,22 @@
     </row>
     <row r="81" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="G81" s="9">
         <v>53.519278</v>
@@ -9079,22 +9094,22 @@
     </row>
     <row r="82" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="G82" s="9">
         <v>53.52115</v>
@@ -9111,22 +9126,22 @@
     </row>
     <row r="83" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="G83" s="9">
         <v>53.522884</v>
@@ -9143,22 +9158,22 @@
     </row>
     <row r="84" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="G84" s="9">
         <v>53.520281</v>
@@ -9175,22 +9190,22 @@
     </row>
     <row r="85" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="G85" s="9">
         <v>53.522781</v>
@@ -9207,22 +9222,22 @@
     </row>
     <row r="86" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="G86" s="9">
         <v>53.52484</v>
@@ -9239,22 +9254,22 @@
     </row>
     <row r="87" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="G87" s="9">
         <v>53.524712</v>
@@ -9271,22 +9286,22 @@
     </row>
     <row r="88" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="B88" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>641</v>
-      </c>
       <c r="F88" s="5" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="G88" s="9">
         <v>53.524751</v>

</xml_diff>

<commit_message>
Leave the starter spreadsheet to repositry/cleanup to avoid a binary merge conflict
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/open-house-content.xlsx
+++ b/content/open-house-content.xlsx
@@ -431,7 +431,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="645">
   <si>
     <t>MEC E Open House website content</t>
   </si>
@@ -610,10 +610,10 @@
     <t>program-presentation</t>
   </si>
   <si>
-    <t>Live program presentation</t>
-  </si>
-  <si>
-    <t>Dr. Nobes presents the Mechanical Engineering program, with remarks from the MEC E Club and the Mechatronics (MCTR) Club.</t>
+    <t>Mechanical Engineering program presentation</t>
+  </si>
+  <si>
+    <t>Learn about the Mechanical Engineering program from the department, with time for questions.</t>
   </si>
   <si>
     <t>10:00</t>
@@ -652,21 +652,6 @@
     <t>2nd and 3rd floors</t>
   </si>
   <si>
-    <t>program-video</t>
-  </si>
-  <si>
-    <t>Rolling program video</t>
-  </si>
-  <si>
-    <t>A short video about the Mechanical Engineering program, playing on a loop. Drop in any time during the building tour.</t>
-  </si>
-  <si>
-    <t>program-room-3-1</t>
-  </si>
-  <si>
-    <t>Room 3-1</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -748,10 +733,10 @@
     <t>stamp-open-house-booth</t>
   </si>
   <si>
-    <t>Live Program Presentation</t>
-  </si>
-  <si>
-    <t>A live presentation by Dr. Nobes on the Mechanical Engineering program, with remarks from the MEC E Club and the Mechatronics (MCTR) Club. 10:00 to 11:00 AM in ETLC E1-001.</t>
+    <t>MEC E Program Presentation</t>
+  </si>
+  <si>
+    <t>Hear from the department about the Mechanical Engineering program, 10:00 to 11:00 AM in ETLC E1-001.</t>
   </si>
   <si>
     <t>E1-001</t>
@@ -760,7 +745,7 @@
     <t>Program Insider</t>
   </si>
   <si>
-    <t>Collected at the live program presentation in ETLC.</t>
+    <t>Collected at the MEC E program presentation.</t>
   </si>
   <si>
     <t>/assets/stamps/program-presentation.svg</t>
@@ -1335,10 +1320,13 @@
     <t>stamp-mctr-club</t>
   </si>
   <si>
+    <t>program-room-3-1</t>
+  </si>
+  <si>
     <t>Room 3-1: MEC E Program Presentation</t>
   </si>
   <si>
-    <t>A short video about the Mechanical Engineering program plays on a loop in Room 3-1. Drop in any time during the building tour.</t>
+    <t>Stop by Room 3-1 during the building tour to learn about the Mechanical Engineering program and ask the department your questions.</t>
   </si>
   <si>
     <t>3-1</t>
@@ -1347,7 +1335,7 @@
     <t>Program Preview</t>
   </si>
   <si>
-    <t>Collected at the program video in Room 3-1.</t>
+    <t>Collected in Room 3-1 on the building tour.</t>
   </si>
   <si>
     <t>/assets/stamps/program-room-3-1.svg</t>
@@ -1437,7 +1425,7 @@
     <t>When and where is the Open House?</t>
   </si>
   <si>
-    <t>Saturday, October 17, 2026, from 9:00 AM to 3:00 PM. Start at the Mechanical Engineering stall in the VVC gym, catch the live program presentation with Dr. Nobes at 10:00 AM in ETLC E1-001, then tour the Mechanical Engineering Building from 11:00 AM to 2:00 PM. The Map page shows the way.</t>
+    <t>Saturday, October 17, 2026, from 9:00 AM to 3:00 PM. Start at the Mechanical Engineering stall in the VVC gym, catch the program presentation at 10:00 AM in ETLC E1-001, then tour the Mechanical Engineering Building from 11:00 AM to 2:00 PM. The Map page shows the way.</t>
   </si>
   <si>
     <t>register</t>
@@ -3047,7 +3035,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K204"/>
+  <dimension ref="A1:K203"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" style="7" customWidth="1"/>
@@ -3197,40 +3185,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>57</v>
-      </c>
+    <row r="5" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="6:11" x14ac:dyDescent="0.25">
       <c r="F6" s="7"/>
@@ -4024,28 +3981,24 @@
       <c r="F203" s="7"/>
       <c r="G203" s="7"/>
     </row>
-    <row r="204" spans="6:11" x14ac:dyDescent="0.25">
-      <c r="F204" s="7"/>
-      <c r="G204" s="7"/>
-    </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" sqref="F10:F204">
+    <dataValidation type="list" allowBlank="1" sqref="F10:F203">
       <formula1>"presentation,tour,booth-fair,food,general"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F204">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F203">
       <formula1>"presentation,tour,booth-fair,food,general"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G10:G204">
+    <dataValidation type="list" allowBlank="1" sqref="G10:G203">
       <formula1>"mece,university"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G204">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G203">
       <formula1>"mece,university"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K10:K204">
+    <dataValidation type="list" allowBlank="1" sqref="K10:K203">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K2:K204">
+    <dataValidation type="list" allowBlank="1" sqref="K2:K203">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4083,61 +4036,61 @@
         <v>39</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>46</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="Q1" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="R1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="S1" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="T1" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="S1" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="T1" s="11" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4145,16 +4098,16 @@
         <v>55</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F2" s="9"/>
       <c r="G2" s="5"/>
@@ -4170,28 +4123,28 @@
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="M2" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="R2" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="T2" s="12" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4199,16 +4152,16 @@
         <v>58</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>63</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="5"/>
@@ -4219,33 +4172,33 @@
         <v>1</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="P3" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="R3" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4253,16 +4206,16 @@
         <v>71</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="5"/>
@@ -4273,7 +4226,7 @@
         <v>2</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="K4" s="9">
         <v>0.236</v>
@@ -4282,45 +4235,45 @@
         <v>0.349</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="P4" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="R4" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="5"/>
@@ -4331,7 +4284,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="K5" s="9">
         <v>0.372</v>
@@ -4340,51 +4293,51 @@
         <v>0.498</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="P5" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="R5" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>34</v>
@@ -4393,7 +4346,7 @@
         <v>3</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="K6" s="9">
         <v>0.805</v>
@@ -4402,49 +4355,49 @@
         <v>0.66</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="P6" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="R6" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="T6" s="12" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>34</v>
@@ -4453,7 +4406,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K7" s="9">
         <v>0.684</v>
@@ -4462,51 +4415,51 @@
         <v>0.763</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="P7" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="R7" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="T7" s="12" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>34</v>
@@ -4515,7 +4468,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K8" s="9">
         <v>0.275</v>
@@ -4524,45 +4477,45 @@
         <v>0.598</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="P8" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="R8" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S8" s="12" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="T8" s="12" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="5"/>
@@ -4573,7 +4526,7 @@
         <v>3</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K9" s="9">
         <v>0.714</v>
@@ -4582,45 +4535,45 @@
         <v>0.491</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="P9" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="R9" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="T9" s="12" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="5"/>
@@ -4631,7 +4584,7 @@
         <v>3</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K10" s="9">
         <v>0.513</v>
@@ -4640,49 +4593,49 @@
         <v>0.67</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="P10" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="R10" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S10" s="12" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="T10" s="12" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="5" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -4691,7 +4644,7 @@
         <v>3</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K11" s="9">
         <v>0.29</v>
@@ -4700,49 +4653,49 @@
         <v>0.566</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="P11" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="R11" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S11" s="12" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="T11" s="12" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>34</v>
@@ -4751,7 +4704,7 @@
         <v>3</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K12" s="9">
         <v>0.159</v>
@@ -4760,51 +4713,51 @@
         <v>0.649</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="P12" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="R12" s="9" t="s">
         <v>30</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="T12" s="12" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>221</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>226</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>34</v>
@@ -4813,7 +4766,7 @@
         <v>3</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K13" s="9">
         <v>0.161</v>
@@ -4822,49 +4775,49 @@
         <v>0.651</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="R13" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S13" s="12" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="T13" s="12" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="5" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>34</v>
@@ -4873,7 +4826,7 @@
         <v>3</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K14" s="9">
         <v>0.245</v>
@@ -4882,45 +4835,45 @@
         <v>0.571</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="P14" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="R14" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S14" s="12" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="T14" s="12" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="5"/>
@@ -4931,7 +4884,7 @@
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="K15" s="9">
         <v>0.153</v>
@@ -4940,49 +4893,49 @@
         <v>0.164</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="P15" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="R15" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S15" s="12" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="T15" s="12" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="5" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>34</v>
@@ -4991,7 +4944,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K16" s="9">
         <v>0.685</v>
@@ -5000,49 +4953,49 @@
         <v>0.758</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P16" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="R16" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S16" s="12" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="T16" s="12" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="5" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>34</v>
@@ -5051,7 +5004,7 @@
         <v>3</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K17" s="9">
         <v>0.285</v>
@@ -5060,49 +5013,49 @@
         <v>0.571</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="R17" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="T17" s="12" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>34</v>
@@ -5111,7 +5064,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K18" s="9">
         <v>0.66</v>
@@ -5120,49 +5073,49 @@
         <v>0.603</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="P18" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="R18" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S18" s="12" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="T18" s="12" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="5" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>34</v>
@@ -5171,7 +5124,7 @@
         <v>3</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="K19" s="9">
         <v>0.233</v>
@@ -5180,45 +5133,45 @@
         <v>0.343</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="P19" s="9" t="s">
         <v>57</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="R19" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S19" s="12" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="T19" s="12" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
     </row>
     <row r="20" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>76</v>
+        <v>295</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>63</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="5"/>
@@ -5229,7 +5182,7 @@
         <v>3</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="K20" s="9">
         <v>0.271</v>
@@ -5238,28 +5191,28 @@
         <v>0.817</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>30</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="R20" s="9" t="s">
         <v>57</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21" spans="3:18" x14ac:dyDescent="0.25">
@@ -5900,7 +5853,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -5908,111 +5861,111 @@
         <v>71</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>76</v>
+        <v>295</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -6043,39 +5996,39 @@
         <v>44</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="H1" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>326</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
@@ -6089,16 +6042,16 @@
     </row>
     <row r="3" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>336</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
@@ -6112,16 +6065,16 @@
     </row>
     <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
@@ -6135,16 +6088,16 @@
     </row>
     <row r="5" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
@@ -6158,23 +6111,23 @@
     </row>
     <row r="6" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>344</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>348</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="5" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>30</v>
@@ -6185,20 +6138,20 @@
     </row>
     <row r="7" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="9" t="s">
@@ -6210,16 +6163,16 @@
     </row>
     <row r="8" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
@@ -6233,16 +6186,16 @@
     </row>
     <row r="9" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
@@ -6256,16 +6209,16 @@
     </row>
     <row r="10" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>362</v>
-      </c>
       <c r="D10" s="5" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
@@ -6279,16 +6232,16 @@
     </row>
     <row r="11" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
@@ -6302,23 +6255,23 @@
     </row>
     <row r="12" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>30</v>
@@ -6329,16 +6282,16 @@
     </row>
     <row r="13" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
@@ -6352,16 +6305,16 @@
     </row>
     <row r="14" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>377</v>
-      </c>
       <c r="D14" s="5" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
@@ -6375,16 +6328,16 @@
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
@@ -6398,16 +6351,16 @@
     </row>
     <row r="16" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
@@ -6421,16 +6374,16 @@
     </row>
     <row r="17" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
@@ -6444,23 +6397,23 @@
     </row>
     <row r="18" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>388</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>392</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>30</v>
@@ -6704,46 +6657,46 @@
         <v>44</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="D1" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="E1" s="8" t="s">
+      <c r="I1" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="J1" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G2" s="9">
         <v>53.523554</v>
@@ -6758,20 +6711,20 @@
     </row>
     <row r="3" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G3" s="9">
         <v>53.521287</v>
@@ -6786,20 +6739,20 @@
     </row>
     <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G4" s="9">
         <v>53.528897</v>
@@ -6814,20 +6767,20 @@
     </row>
     <row r="5" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G5" s="9">
         <v>53.526203</v>
@@ -6842,20 +6795,20 @@
     </row>
     <row r="6" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G6" s="9">
         <v>53.52527</v>
@@ -6870,20 +6823,20 @@
     </row>
     <row r="7" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G7" s="9">
         <v>53.525312</v>
@@ -6898,20 +6851,20 @@
     </row>
     <row r="8" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G8" s="9">
         <v>53.528827</v>
@@ -6926,20 +6879,20 @@
     </row>
     <row r="9" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="G9" s="9">
         <v>53.525374</v>
@@ -6954,20 +6907,20 @@
     </row>
     <row r="10" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="G10" s="9">
         <v>53.52575</v>
@@ -6982,20 +6935,20 @@
     </row>
     <row r="11" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="G11" s="9">
         <v>53.526227</v>
@@ -7010,20 +6963,20 @@
     </row>
     <row r="12" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="G12" s="9">
         <v>53.521933</v>
@@ -7038,20 +6991,20 @@
     </row>
     <row r="13" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="G13" s="9">
         <v>53.526054</v>
@@ -7066,20 +7019,20 @@
     </row>
     <row r="14" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="G14" s="9">
         <v>53.527982</v>
@@ -7094,20 +7047,20 @@
     </row>
     <row r="15" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="G15" s="9">
         <v>53.526848</v>
@@ -7122,20 +7075,20 @@
     </row>
     <row r="16" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="G16" s="9">
         <v>53.518596</v>
@@ -7150,20 +7103,20 @@
     </row>
     <row r="17" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="G17" s="9">
         <v>53.525281</v>
@@ -7178,20 +7131,20 @@
     </row>
     <row r="18" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="G18" s="9">
         <v>53.526405</v>
@@ -7206,20 +7159,20 @@
     </row>
     <row r="19" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G19" s="9">
         <v>53.526452</v>
@@ -7236,20 +7189,20 @@
     </row>
     <row r="20" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G20" s="9">
         <v>53.520234</v>
@@ -7266,20 +7219,20 @@
     </row>
     <row r="21" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G21" s="9">
         <v>53.526721</v>
@@ -7296,20 +7249,20 @@
     </row>
     <row r="22" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G22" s="9">
         <v>53.522632</v>
@@ -7326,20 +7279,20 @@
     </row>
     <row r="23" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G23" s="9">
         <v>53.520485</v>
@@ -7356,20 +7309,20 @@
     </row>
     <row r="24" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G24" s="9">
         <v>53.526051</v>
@@ -7386,20 +7339,20 @@
     </row>
     <row r="25" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G25" s="9">
         <v>53.526912</v>
@@ -7416,20 +7369,20 @@
     </row>
     <row r="26" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G26" s="9">
         <v>53.519489</v>
@@ -7446,20 +7399,20 @@
     </row>
     <row r="27" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G27" s="9">
         <v>53.526097</v>
@@ -7476,20 +7429,20 @@
     </row>
     <row r="28" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G28" s="9">
         <v>53.522735</v>
@@ -7506,20 +7459,20 @@
     </row>
     <row r="29" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G29" s="9">
         <v>53.523398</v>
@@ -7536,20 +7489,20 @@
     </row>
     <row r="30" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G30" s="9">
         <v>53.526831</v>
@@ -7566,20 +7519,20 @@
     </row>
     <row r="31" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G31" s="9">
         <v>53.522498</v>
@@ -7596,20 +7549,20 @@
     </row>
     <row r="32" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G32" s="9">
         <v>53.521206</v>
@@ -7626,20 +7579,20 @@
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G33" s="9">
         <v>53.526778</v>
@@ -7656,20 +7609,20 @@
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G34" s="9">
         <v>53.521769</v>
@@ -7686,20 +7639,20 @@
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G35" s="9">
         <v>53.527243</v>
@@ -7716,20 +7669,20 @@
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G36" s="9">
         <v>53.526834</v>
@@ -7746,20 +7699,20 @@
     </row>
     <row r="37" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G37" s="9">
         <v>53.521291</v>
@@ -7776,20 +7729,20 @@
     </row>
     <row r="38" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G38" s="9">
         <v>53.526281</v>
@@ -7806,20 +7759,20 @@
     </row>
     <row r="39" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G39" s="9">
         <v>53.527298</v>
@@ -7836,20 +7789,20 @@
     </row>
     <row r="40" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G40" s="9">
         <v>53.526922</v>
@@ -7866,20 +7819,20 @@
     </row>
     <row r="41" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G41" s="9">
         <v>53.525208</v>
@@ -7896,20 +7849,20 @@
     </row>
     <row r="42" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G42" s="9">
         <v>53.527654</v>
@@ -7926,20 +7879,20 @@
     </row>
     <row r="43" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G43" s="9">
         <v>53.529014</v>
@@ -7956,20 +7909,20 @@
     </row>
     <row r="44" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G44" s="9">
         <v>53.521611</v>
@@ -7986,20 +7939,20 @@
     </row>
     <row r="45" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G45" s="9">
         <v>53.521595</v>
@@ -8016,20 +7969,20 @@
     </row>
     <row r="46" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G46" s="9">
         <v>53.520763</v>
@@ -8046,20 +7999,20 @@
     </row>
     <row r="47" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G47" s="9">
         <v>53.526621</v>
@@ -8076,20 +8029,20 @@
     </row>
     <row r="48" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G48" s="9">
         <v>53.521375</v>
@@ -8106,20 +8059,20 @@
     </row>
     <row r="49" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G49" s="9">
         <v>53.525055</v>
@@ -8136,20 +8089,20 @@
     </row>
     <row r="50" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G50" s="9">
         <v>53.522628</v>
@@ -8166,20 +8119,20 @@
     </row>
     <row r="51" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G51" s="9">
         <v>53.52057</v>
@@ -8196,20 +8149,20 @@
     </row>
     <row r="52" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="G52" s="9">
         <v>53.527441</v>
@@ -8226,20 +8179,20 @@
     </row>
     <row r="53" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G53" s="9">
         <v>53.521685</v>
@@ -8256,20 +8209,20 @@
     </row>
     <row r="54" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="G54" s="9">
         <v>53.52063</v>
@@ -8286,20 +8239,20 @@
     </row>
     <row r="55" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G55" s="9">
         <v>53.52495</v>
@@ -8314,20 +8267,20 @@
     </row>
     <row r="56" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="G56" s="9">
         <v>53.52455</v>
@@ -8342,20 +8295,20 @@
     </row>
     <row r="57" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="G57" s="9">
         <v>53.51885</v>
@@ -8370,20 +8323,20 @@
     </row>
     <row r="58" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="G58" s="9">
         <v>53.52735</v>
@@ -8398,20 +8351,20 @@
     </row>
     <row r="59" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="G59" s="9">
         <v>53.520064</v>
@@ -8426,20 +8379,20 @@
     </row>
     <row r="60" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C60" s="5"/>
       <c r="D60" s="5" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="G60" s="9">
         <v>53.52485</v>
@@ -8454,22 +8407,22 @@
     </row>
     <row r="61" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>544</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="F61" s="5" t="s">
         <v>546</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>547</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>548</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>549</v>
-      </c>
-      <c r="F61" s="5" t="s">
-        <v>550</v>
       </c>
       <c r="G61" s="9">
         <v>53.524907</v>
@@ -8486,22 +8439,22 @@
     </row>
     <row r="62" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="G62" s="9">
         <v>53.524349</v>
@@ -8518,22 +8471,22 @@
     </row>
     <row r="63" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="G63" s="9">
         <v>53.522853</v>
@@ -8550,22 +8503,22 @@
     </row>
     <row r="64" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="G64" s="9">
         <v>53.522936</v>
@@ -8582,22 +8535,22 @@
     </row>
     <row r="65" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="G65" s="9">
         <v>53.522841</v>
@@ -8614,22 +8567,22 @@
     </row>
     <row r="66" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="G66" s="9">
         <v>53.527555</v>
@@ -8646,22 +8599,22 @@
     </row>
     <row r="67" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="G67" s="9">
         <v>53.526058</v>
@@ -8678,22 +8631,22 @@
     </row>
     <row r="68" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="G68" s="9">
         <v>53.520408</v>
@@ -8710,22 +8663,22 @@
     </row>
     <row r="69" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="G69" s="9">
         <v>53.521436</v>
@@ -8742,22 +8695,22 @@
     </row>
     <row r="70" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="G70" s="9">
         <v>53.520333</v>
@@ -8774,22 +8727,22 @@
     </row>
     <row r="71" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="G71" s="9">
         <v>53.522316</v>
@@ -8806,22 +8759,22 @@
     </row>
     <row r="72" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D72" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>585</v>
+      </c>
+      <c r="F72" s="5" t="s">
         <v>588</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>589</v>
-      </c>
-      <c r="F72" s="5" t="s">
-        <v>592</v>
       </c>
       <c r="G72" s="9">
         <v>53.522998</v>
@@ -8838,22 +8791,22 @@
     </row>
     <row r="73" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="G73" s="9">
         <v>53.519823</v>
@@ -8870,22 +8823,22 @@
     </row>
     <row r="74" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D74" s="5" t="s">
+        <v>590</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>591</v>
+      </c>
+      <c r="F74" s="5" t="s">
         <v>594</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>595</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>598</v>
       </c>
       <c r="G74" s="9">
         <v>53.518952</v>
@@ -8902,22 +8855,22 @@
     </row>
     <row r="75" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="G75" s="9">
         <v>53.521462</v>
@@ -8934,22 +8887,22 @@
     </row>
     <row r="76" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="G76" s="9">
         <v>53.522356</v>
@@ -8966,22 +8919,22 @@
     </row>
     <row r="77" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D77" s="5" t="s">
+        <v>600</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="F77" s="5" t="s">
         <v>604</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="F77" s="5" t="s">
-        <v>608</v>
       </c>
       <c r="G77" s="9">
         <v>53.523026</v>
@@ -8998,22 +8951,22 @@
     </row>
     <row r="78" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>611</v>
+        <v>607</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="G78" s="9">
         <v>53.524645</v>
@@ -9030,22 +8983,22 @@
     </row>
     <row r="79" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="G79" s="9">
         <v>53.522775</v>
@@ -9062,22 +9015,22 @@
     </row>
     <row r="80" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D80" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="F80" s="5" t="s">
         <v>614</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>615</v>
-      </c>
-      <c r="F80" s="5" t="s">
-        <v>618</v>
       </c>
       <c r="G80" s="9">
         <v>53.523038</v>
@@ -9094,22 +9047,22 @@
     </row>
     <row r="81" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="G81" s="9">
         <v>53.519278</v>
@@ -9126,22 +9079,22 @@
     </row>
     <row r="82" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="G82" s="9">
         <v>53.52115</v>
@@ -9158,22 +9111,22 @@
     </row>
     <row r="83" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="G83" s="9">
         <v>53.522884</v>
@@ -9190,22 +9143,22 @@
     </row>
     <row r="84" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="G84" s="9">
         <v>53.520281</v>
@@ -9222,22 +9175,22 @@
     </row>
     <row r="85" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="G85" s="9">
         <v>53.522781</v>
@@ -9254,22 +9207,22 @@
     </row>
     <row r="86" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="G86" s="9">
         <v>53.52484</v>
@@ -9286,22 +9239,22 @@
     </row>
     <row r="87" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="G87" s="9">
         <v>53.524712</v>
@@ -9318,22 +9271,22 @@
     </row>
     <row r="88" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D88" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="F88" s="5" t="s">
         <v>644</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>645</v>
-      </c>
-      <c r="F88" s="5" t="s">
-        <v>648</v>
       </c>
       <c r="G88" s="9">
         <v>53.524751</v>

</xml_diff>